<commit_message>
Sprint sheet: T12 to T16 done, G3 in progress
G3 stays in progress until the live kill, alert, restart sequence has passed twice in a row.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FunnelStream-Sprint-Plan-v3.xlsx
+++ b/docs/FunnelStream-Sprint-Plan-v3.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -2667,7 +2667,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
@@ -2771,12 +2770,6 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3082,7 +3075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5368,22 +5361,6 @@
         <v/>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
   </sheetData>
   <conditionalFormatting sqref="D4:M44">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">

</xml_diff>

<commit_message>
Add the inventory design spec and update the sprint sheet
The spec describes one platform for two users: live inventory and traffic for
operations, and the D-1 campaign and sales view for marketing, with estimated
ad spend exposed to out-of-stock products as the bridge. It was reviewed by a
data engineer and a business manager.

The sprint sheet gets the rows SPD, ALR and INV0-INV6, new notes for G1, G2,
G3, T17 and DOC, and a fix for Hours Done % (it divided tasks by hours).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FunnelStream-Sprint-Plan-v3.xlsx
+++ b/docs/FunnelStream-Sprint-Plan-v3.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Status as of Thursday 8 October 2026. Dates of Done tasks are actual (commit history); dates of open tasks are planned.</t>
+          <t>Status as of Saturday 10 October 2026. Dates of Done tasks are actual (commit history); dates of open tasks are planned.</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Review fixes done; full Docker suite re-run pending</t>
+          <t>Review fixes done; G1 Spark tests 10 of 10 again after SPD (10 Oct)</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Live check: 14 panels, all rules fired</t>
+          <t>Live check: 14 panels, all rules fired; 10 Oct: heartbeat rule added (ALR)</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2224,35 +2224,35 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>SPD</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Failure demo with Grafana: kill Silver, alert, restart, no duplicates</t>
+          <t>Silver and live sink speed-up: concurrent MERGEs, concurrent sink compute, job-group inheritance</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Member 5</t>
+          <t>Member 2</t>
         </is>
       </c>
       <c r="D36" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="E36" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="F36" s="3">
         <f>E36-D36+1</f>
         <v/>
       </c>
       <c r="G36" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>G2, T16</t>
+          <t>T8, G1</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Best live moment for the defense</t>
+          <t>Batch plus sink about 50-70 s to about 25 s; tests first; expert review done; uncommitted until you say</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2274,12 +2274,12 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>ALR</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Samples, benchmark, README</t>
+          <t>Alert redesign: heartbeat rule (2 min), no-events widened to 5 min</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2288,21 +2288,21 @@
         </is>
       </c>
       <c r="D37" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="E37" s="17" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="F37" s="3">
         <f>E37-D37+1</f>
         <v/>
       </c>
       <c r="G37" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>T8, T10c</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2312,47 +2312,47 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Run 1-2M events once</t>
+          <t>4 rules provisioned; the old 2-minute rule could not stay quiet at a 60 s batch cycle</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>T18</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Power BI model and pages (Campaign and Funnel first)</t>
+          <t>Failure demo with Grafana: kill Silver, alert, restart, no duplicates</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Member 1</t>
+          <t>Member 5</t>
         </is>
       </c>
       <c r="D38" s="17" t="n">
         <v>46306</v>
       </c>
       <c r="E38" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F38" s="3">
         <f>E38-D38+1</f>
         <v/>
       </c>
       <c r="G38" s="6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>T10c, T12</t>
+          <t>G2, T16, ALR, SPD</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2362,33 +2362,33 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Read-only token; extra pages only if time</t>
+          <t>Code done. Not passed twice yet: the 60 s Silver batch made the 2-minute alert flap; SPD and ALR fix that, then run twice</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Customer 360 table and page (STRETCH)</t>
+          <t>Samples, benchmark, README</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Member 4</t>
+          <t>Member 5</t>
         </is>
       </c>
       <c r="D39" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="E39" s="17" t="n">
         <v>46307</v>
@@ -2398,21 +2398,21 @@
         <v/>
       </c>
       <c r="G39" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T8, T10c, SPD</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Stretch</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Cut first if late</t>
+          <t>End-to-end benchmark, 1 to 2M events, run once after SPD; samples from Gold; README</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2424,21 +2424,21 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>T18</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Refresh PDF, deck, README screenshots</t>
+          <t>Power BI model and pages (Campaign and Funnel first)</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Member 5</t>
+          <t>Member 1</t>
         </is>
       </c>
       <c r="D40" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="E40" s="17" t="n">
         <v>46307</v>
@@ -2448,11 +2448,11 @@
         <v/>
       </c>
       <c r="G40" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>G3, T18</t>
+          <t>T10c, T12</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Documents are still from 5 Oct</t>
+          <t>Read-only token; extra pages only if time</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2474,145 +2474,145 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Integration: Kafka to Silver to Postgres/Grafana and Databricks Gold</t>
+          <t>Customer 360 table and page (STRETCH)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Member 4</t>
         </is>
       </c>
       <c r="D41" s="17" t="n">
-        <v>46303</v>
+        <v>46307</v>
       </c>
       <c r="E41" s="17" t="n">
-        <v>46303</v>
+        <v>46307</v>
       </c>
       <c r="F41" s="3">
         <f>E41-D41+1</f>
         <v/>
       </c>
       <c r="G41" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>T10c, G1</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Stretch</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Verified live on 8 Oct</t>
+          <t>Cut first if late</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To do</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>INV0</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Failure demo, 1-2M run, benchmark recorded</t>
+          <t>Spec: live inventory for operations and D-1 marketing</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Member 5</t>
         </is>
       </c>
       <c r="D42" s="17" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="E42" s="17" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="F42" s="3">
         <f>E42-D42+1</f>
         <v/>
       </c>
       <c r="G42" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>G3, T17</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Team session</t>
+          <t>Spec in docs/superpowers/specs; reviewed by a data engineer and a business manager; owner review pending</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>INV1</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Rehearsal, final deck and PDF check</t>
+          <t>Inventory contract: stock events, validator, transform, topic</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Member 2</t>
         </is>
       </c>
       <c r="D43" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="E43" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F43" s="3">
         <f>E43-D43+1</f>
         <v/>
       </c>
       <c r="G43" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>M2, DOC</t>
+          <t>INV0, T2</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Milestone</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Share links from Share menu</t>
+          <t>Standard envelope with payload; explicit stock branch; tests first</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2624,149 +2624,623 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>INV2</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Defense</t>
+          <t>Simulator stock ledger and hero stock-out scenario</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Member 1</t>
         </is>
       </c>
       <c r="D44" s="17" t="n">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="E44" s="17" t="n">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="F44" s="3">
         <f>E44-D44+1</f>
         <v/>
       </c>
       <c r="G44" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>INV1</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Seeded, never negative, 8 stores, oversold lines recorded</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>INV3</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Bronze and Silver stock tables, DDL, count-pinned tests</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Member 2</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E45" s="17" t="n">
+        <v>46306</v>
+      </c>
+      <c r="F45" s="3">
+        <f>E45-D45+1</f>
+        <v/>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>INV1, SPD</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Adds MERGEs to a batch that SPD made faster</t>
+        </is>
+      </c>
+      <c r="K45" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>INV4</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Live stock tables in Postgres and the sink recompute</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Member 3</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E46" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F46" s="3">
+        <f>E46-D46+1</f>
+        <v/>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>INV3, G1</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>live_stock_now, live_oos_demand_minute, dim_store</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>INV5</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Grafana: Operations live inventory dashboard and out-of-stock demand alert</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Member 5</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E47" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F47" s="3">
+        <f>E47-D47+1</f>
+        <v/>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>INV4</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>7 panels, one alert</t>
+        </is>
+      </c>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>INV6</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Marketing D-1 mart in Postgres and Grafana page (estimated exposed spend)</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Member 4</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E48" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F48" s="3">
+        <f>E48-D48+1</f>
+        <v/>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>INV4, T12</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>Cut first among the inventory rows</t>
+        </is>
+      </c>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>DOC</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Refresh PDF, deck, README screenshots</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Member 5</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E49" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F49" s="3">
+        <f>E49-D49+1</f>
+        <v/>
+      </c>
+      <c r="G49" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>G3, T18</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>Documents are still from 5 Oct; add the alert redesign and the inventory story</t>
+        </is>
+      </c>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Integration: Kafka to Silver to Postgres/Grafana and Databricks Gold</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E50" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="F50" s="3">
+        <f>E50-D50+1</f>
+        <v/>
+      </c>
+      <c r="G50" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>T10c, G1</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>Verified live on 8 Oct</t>
+        </is>
+      </c>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Failure demo, 1-2M run, benchmark recorded</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E51" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F51" s="3">
+        <f>E51-D51+1</f>
+        <v/>
+      </c>
+      <c r="G51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>G3, T17</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>Team session</t>
+        </is>
+      </c>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="I44" s="3" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Rehearsal, final deck and PDF check</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E52" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F52" s="3">
+        <f>E52-D52+1</f>
+        <v/>
+      </c>
+      <c r="G52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>M2, DOC</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="J44" s="4" t="n"/>
-      <c r="K44" s="6" t="inlineStr">
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>Share links from Share menu</t>
+        </is>
+      </c>
+      <c r="K52" s="6" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Defense</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E53" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F53" s="3">
+        <f>E53-D53+1</f>
+        <v/>
+      </c>
+      <c r="G53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="n"/>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>Assumptions</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>Productive hours per member per day: 6 (blue input on Team Load sheet).</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B57" s="8" t="inlineStr">
         <is>
           <t>Hours are focused build time, not calendar time. Hours of Done tasks are the original estimates, not measured time. Integration and milestone rows (owner All) carry no hours and are excluded from Team Load.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>Blue text = inputs you can change. Black = formulas.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B59" s="8" t="inlineStr">
         <is>
           <t>T19 is stretch: drop it first. Cut order after that: rec_product and customer_360, the SQL checks beyond the five key ones, Power BI pages beyond Campaign and Funnel. Never cut: attribution (T13), campaign summaries (T12), Grafana (G2) and the failure demo (G3).</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>Spark runs in Docker (Python 3.11 and Java 17 are inside the image); the host needs Python 3.11 only. Status column is an input (blue): Done, In progress, To do.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>6.</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B61" s="8" t="inlineStr">
         <is>
           <t>T0 was a human step: Databricks workspace, SQL warehouse and token. The token stays in .env only.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>7.</t>
         </is>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>Decision date 10 Oct: batch entry point is a Python script (T15). The Airflow DAG exists for the daily ad report only.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
         <is>
           <t>8.</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B63" s="8" t="inlineStr">
         <is>
           <t>Tasks C1-C4, AD, D1, D2, DEMO, G1, G2 were added after the 4 Oct plan (external review, address and tracking URL, live monitoring).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>9.</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>10 Oct: rows SPD, ALR and INV0-INV6 were added after the speed measurements and the inventory spec. Hours of these rows are estimates and owners follow the area precedent; change them freely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>10.</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Inventory cut order: INV6 first, then the INV5 alert, then the INV5 dashboard polish. Keep INV1-INV4 and a basic dashboard. The inventory data is simulated and is labeled as simulated.</t>
         </is>
       </c>
     </row>
@@ -2858,11 +3332,11 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$44,A4)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A4)</f>
         <v/>
       </c>
       <c r="C4" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$44,A4,'Sprint Plan'!$G$4:$G$44)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A4,'Sprint Plan'!$G$4:$G$53)</f>
         <v/>
       </c>
       <c r="D4" s="12">
@@ -2885,11 +3359,11 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$44,A5)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$44,A5,'Sprint Plan'!$G$4:$G$44)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A5,'Sprint Plan'!$G$4:$G$53)</f>
         <v/>
       </c>
       <c r="D5" s="12">
@@ -2917,11 +3391,11 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$44,A6)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$44,A6,'Sprint Plan'!$G$4:$G$44)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A6,'Sprint Plan'!$G$4:$G$53)</f>
         <v/>
       </c>
       <c r="D6" s="12">
@@ -2942,7 +3416,7 @@
         </is>
       </c>
       <c r="I6" s="18">
-        <f>COUNTIF('Sprint Plan'!$K$4:$K$44,"Done")</f>
+        <f>COUNTIF('Sprint Plan'!$K$4:$K$53,"Done")</f>
         <v/>
       </c>
     </row>
@@ -2953,11 +3427,11 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$44,A7)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$44,A7,'Sprint Plan'!$G$4:$G$44)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A7,'Sprint Plan'!$G$4:$G$53)</f>
         <v/>
       </c>
       <c r="D7" s="12">
@@ -2978,7 +3452,7 @@
         </is>
       </c>
       <c r="I7" s="18">
-        <f>COUNTIF('Sprint Plan'!$K$4:$K$44,"In progress")</f>
+        <f>COUNTIF('Sprint Plan'!$K$4:$K$53,"In progress")</f>
         <v/>
       </c>
     </row>
@@ -2989,11 +3463,11 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$44,A8)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$44,A8,'Sprint Plan'!$G$4:$G$44)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A8,'Sprint Plan'!$G$4:$G$53)</f>
         <v/>
       </c>
       <c r="D8" s="12">
@@ -3014,7 +3488,7 @@
         </is>
       </c>
       <c r="I8" s="18">
-        <f>COUNTIF('Sprint Plan'!$K$4:$K$44,"To do")</f>
+        <f>COUNTIF('Sprint Plan'!$K$4:$K$53,"To do")</f>
         <v/>
       </c>
     </row>
@@ -3038,7 +3512,7 @@
         </is>
       </c>
       <c r="I9" s="18">
-        <f>SUMIF('Sprint Plan'!$K$4:$K$44,"Done",'Sprint Plan'!$G$4:$G$44)</f>
+        <f>SUMIF('Sprint Plan'!$K$4:$K$53,"Done",'Sprint Plan'!$G$4:$G$53)</f>
         <v/>
       </c>
     </row>
@@ -3049,7 +3523,7 @@
         </is>
       </c>
       <c r="I10" s="18">
-        <f>SUM('Sprint Plan'!$G$4:$G$44)</f>
+        <f>SUM('Sprint Plan'!$G$4:$G$53)</f>
         <v/>
       </c>
     </row>
@@ -3060,7 +3534,7 @@
         </is>
       </c>
       <c r="I11" s="19">
-        <f>I8/I9</f>
+        <f>I9/I10</f>
         <v/>
       </c>
     </row>
@@ -3075,7 +3549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5361,8 +5835,494 @@
         <v/>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="8">
+        <f>'Sprint Plan'!A45</f>
+        <v/>
+      </c>
+      <c r="B45" s="8">
+        <f>'Sprint Plan'!B45</f>
+        <v/>
+      </c>
+      <c r="C45" s="8">
+        <f>'Sprint Plan'!C45</f>
+        <v/>
+      </c>
+      <c r="D45" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D45,D$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="E45" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D45,E$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="F45" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D45,F$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="G45" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D45,G$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="H45" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D45,H$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="I45" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D45,I$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="J45" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D45,J$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="K45" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D45,K$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="L45" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D45,L$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+      <c r="M45" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D45,M$3&lt;='Sprint Plan'!$E45),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8">
+        <f>'Sprint Plan'!A46</f>
+        <v/>
+      </c>
+      <c r="B46" s="8">
+        <f>'Sprint Plan'!B46</f>
+        <v/>
+      </c>
+      <c r="C46" s="8">
+        <f>'Sprint Plan'!C46</f>
+        <v/>
+      </c>
+      <c r="D46" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D46,D$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="E46" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D46,E$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="F46" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D46,F$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="G46" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D46,G$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="H46" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D46,H$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="I46" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D46,I$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="J46" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D46,J$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="K46" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D46,K$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="L46" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D46,L$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+      <c r="M46" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D46,M$3&lt;='Sprint Plan'!$E46),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8">
+        <f>'Sprint Plan'!A47</f>
+        <v/>
+      </c>
+      <c r="B47" s="8">
+        <f>'Sprint Plan'!B47</f>
+        <v/>
+      </c>
+      <c r="C47" s="8">
+        <f>'Sprint Plan'!C47</f>
+        <v/>
+      </c>
+      <c r="D47" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D47,D$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="E47" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D47,E$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="F47" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D47,F$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D47,G$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="H47" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D47,H$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="I47" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D47,I$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="J47" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D47,J$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="K47" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D47,K$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="L47" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D47,L$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+      <c r="M47" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D47,M$3&lt;='Sprint Plan'!$E47),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8">
+        <f>'Sprint Plan'!A48</f>
+        <v/>
+      </c>
+      <c r="B48" s="8">
+        <f>'Sprint Plan'!B48</f>
+        <v/>
+      </c>
+      <c r="C48" s="8">
+        <f>'Sprint Plan'!C48</f>
+        <v/>
+      </c>
+      <c r="D48" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D48,D$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="E48" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D48,E$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D48,F$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="G48" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D48,G$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="H48" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D48,H$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="I48" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D48,I$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="J48" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D48,J$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="K48" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D48,K$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="L48" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D48,L$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+      <c r="M48" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D48,M$3&lt;='Sprint Plan'!$E48),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8">
+        <f>'Sprint Plan'!A49</f>
+        <v/>
+      </c>
+      <c r="B49" s="8">
+        <f>'Sprint Plan'!B49</f>
+        <v/>
+      </c>
+      <c r="C49" s="8">
+        <f>'Sprint Plan'!C49</f>
+        <v/>
+      </c>
+      <c r="D49" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D49,D$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="E49" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D49,E$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D49,F$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="G49" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D49,G$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="H49" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D49,H$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="I49" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D49,I$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="J49" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D49,J$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="K49" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D49,K$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="L49" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D49,L$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+      <c r="M49" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D49,M$3&lt;='Sprint Plan'!$E49),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8">
+        <f>'Sprint Plan'!A50</f>
+        <v/>
+      </c>
+      <c r="B50" s="8">
+        <f>'Sprint Plan'!B50</f>
+        <v/>
+      </c>
+      <c r="C50" s="8">
+        <f>'Sprint Plan'!C50</f>
+        <v/>
+      </c>
+      <c r="D50" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D50,D$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="E50" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D50,E$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="F50" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D50,F$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D50,G$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="H50" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D50,H$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="I50" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D50,I$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="J50" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D50,J$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="K50" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D50,K$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="L50" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D50,L$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+      <c r="M50" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D50,M$3&lt;='Sprint Plan'!$E50),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8">
+        <f>'Sprint Plan'!A51</f>
+        <v/>
+      </c>
+      <c r="B51" s="8">
+        <f>'Sprint Plan'!B51</f>
+        <v/>
+      </c>
+      <c r="C51" s="8">
+        <f>'Sprint Plan'!C51</f>
+        <v/>
+      </c>
+      <c r="D51" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D51,D$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="E51" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D51,E$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D51,F$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D51,G$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="H51" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D51,H$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="I51" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D51,I$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="J51" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D51,J$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="K51" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D51,K$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="L51" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D51,L$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+      <c r="M51" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D51,M$3&lt;='Sprint Plan'!$E51),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8">
+        <f>'Sprint Plan'!A52</f>
+        <v/>
+      </c>
+      <c r="B52" s="8">
+        <f>'Sprint Plan'!B52</f>
+        <v/>
+      </c>
+      <c r="C52" s="8">
+        <f>'Sprint Plan'!C52</f>
+        <v/>
+      </c>
+      <c r="D52" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D52,D$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="E52" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D52,E$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="F52" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D52,F$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="G52" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D52,G$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="H52" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D52,H$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="I52" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D52,I$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="J52" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D52,J$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="K52" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D52,K$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="L52" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D52,L$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+      <c r="M52" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D52,M$3&lt;='Sprint Plan'!$E52),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8">
+        <f>'Sprint Plan'!A53</f>
+        <v/>
+      </c>
+      <c r="B53" s="8">
+        <f>'Sprint Plan'!B53</f>
+        <v/>
+      </c>
+      <c r="C53" s="8">
+        <f>'Sprint Plan'!C53</f>
+        <v/>
+      </c>
+      <c r="D53" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D53,D$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="E53" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D53,E$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="F53" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D53,F$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="G53" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D53,G$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="H53" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D53,H$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="I53" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D53,I$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="J53" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D53,J$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="K53" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D53,K$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="L53" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D53,L$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+      <c r="M53" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D53,M$3&lt;='Sprint Plan'!$E53),1,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D4:M44">
+  <conditionalFormatting sqref="D4:M53">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(D4=1,LEFT($A4,1)="M")</formula>
     </cfRule>

</xml_diff>

<commit_message>
Update the handoff, the running guide, the inventory spec and plan, the sprint sheet and add the data model review
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FunnelStream-Sprint-Plan-v3.xlsx
+++ b/docs/FunnelStream-Sprint-Plan-v3.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2262,12 +2262,12 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Batch plus sink about 50-70 s to about 25 s; tests first; expert review done; uncommitted until you say</t>
+          <t>Batch plus sink about 50-70 s to about 22 s; committed 35c7f64; expert review done</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2338,10 +2338,10 @@
         </is>
       </c>
       <c r="D38" s="17" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E38" s="17" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="F38" s="3">
         <f>E38-D38+1</f>
@@ -2362,12 +2362,12 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Code done. Not passed twice yet: the 60 s Silver batch made the 2-minute alert flap; SPD and ALR fix that, then run twice</t>
+          <t>Parked 10 Oct: two attempts ended when the Docker WSL VM restarted (21:52 and 22:05) and the PC clock jumped days on sleep and resume. Code, speed and alerts are done. Retry Mon 12 Oct after the PC checks; fallback: a recorded run plus the Spark replay tests</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>To do</t>
         </is>
       </c>
     </row>
@@ -2412,12 +2412,12 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>End-to-end benchmark, 1 to 2M events, run once after SPD; samples from Gold; README</t>
+          <t>Samples and README done and verified; benchmark script verified, real run pending (recreates Kafka)</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Read-only token; extra pages only if time</t>
+          <t>Power BI Desktop downloading; model v2 with inventory and express pages in dashboards/powerbi (MODEL.md, measures.dax)</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Spec in docs/superpowers/specs; reviewed by a data engineer and a business manager; owner review pending</t>
+          <t>Spec approved; sections 1 to 13 incl. Power BI, daily Grafana insights and the 20-minute express promise</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Seeded, never negative, 8 stores, oversold lines recorded</t>
+          <t>Seeded, never negative, 8 stores, oversold lines recorded; express orders in INV8a</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2874,21 +2874,21 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>INV7</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Refresh PDF, deck, README screenshots</t>
+          <t>Daily inventory mart, Grafana inventory-insights page, Power BI tables</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Member 5</t>
+          <t>Member 3</t>
         </is>
       </c>
       <c r="D49" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="E49" s="17" t="n">
         <v>46307</v>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>G3, T18</t>
+          <t>INV4</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>Documents are still from 5 Oct; add the alert redesign and the inventory story</t>
+          <t>inventory_daily, oos_demand_daily, express_daily; second Grafana dashboard; Power BI reads the same tables</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -2924,67 +2924,67 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>INV8a</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Integration: Kafka to Silver to Postgres/Grafana and Databricks Gold</t>
+          <t>Express orders and the 20-minute promise: contract, Silver table, simulator</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Member 1</t>
         </is>
       </c>
       <c r="D50" s="17" t="n">
-        <v>46303</v>
+        <v>46306</v>
       </c>
       <c r="E50" s="17" t="n">
-        <v>46303</v>
+        <v>46306</v>
       </c>
       <c r="F50" s="3">
         <f>E50-D50+1</f>
         <v/>
       </c>
       <c r="G50" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>T10c, G1</t>
+          <t>INV2</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>Verified live on 8 Oct</t>
+          <t>service and promised_minutes on the order; express orders take 8 to 17.5 min and never over 19.5; noise protected</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To do</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>INV8b</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Failure demo, 1-2M run, benchmark recorded</t>
+          <t>Live express SLA table, Grafana panels and the any-breach alert</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Member 5</t>
         </is>
       </c>
       <c r="D51" s="17" t="n">
@@ -2998,21 +2998,21 @@
         <v/>
       </c>
       <c r="G51" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>G3, T17</t>
+          <t>INV4, INV8a</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>Team session</t>
+          <t>fs-express-sla fires on any breach; rehearsal flags shorten the promise and make every Kth order late</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -3024,17 +3024,17 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>DOC</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Rehearsal, final deck and PDF check</t>
+          <t>Refresh PDF, deck, README screenshots</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Member 5</t>
         </is>
       </c>
       <c r="D52" s="17" t="n">
@@ -3048,21 +3048,21 @@
         <v/>
       </c>
       <c r="G52" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>M2, DOC</t>
+          <t>G3, T18</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Milestone</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>Share links from Share menu</t>
+          <t>Documents are still from 5 Oct; add the alert redesign and the inventory story</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -3074,12 +3074,12 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Defense</t>
+          <t>Integration: Kafka to Silver to Postgres/Grafana and Databricks Gold</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -3088,10 +3088,10 @@
         </is>
       </c>
       <c r="D53" s="17" t="n">
-        <v>46308</v>
+        <v>46303</v>
       </c>
       <c r="E53" s="17" t="n">
-        <v>46308</v>
+        <v>46303</v>
       </c>
       <c r="F53" s="3">
         <f>E53-D53+1</f>
@@ -3102,148 +3102,331 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
+          <t>T10c, G1</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>Verified live on 8 Oct</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Failure demo, 1-2M run, benchmark recorded</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E54" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F54" s="3">
+        <f>E54-D54+1</f>
+        <v/>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>G3, T17</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>Team session</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="I53" s="3" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Rehearsal, final deck and PDF check</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E55" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F55" s="3">
+        <f>E55-D55+1</f>
+        <v/>
+      </c>
+      <c r="G55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>M2, DOC</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="J53" s="4" t="n"/>
-      <c r="K53" s="6" t="inlineStr">
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>Share links from Share menu</t>
+        </is>
+      </c>
+      <c r="K55" s="6" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="7" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Defense</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E56" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F56" s="3">
+        <f>E56-D56+1</f>
+        <v/>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="n"/>
+      <c r="K56" s="6" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>Assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>Productive hours per member per day: 6 (blue input on Team Load sheet).</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>Hours are focused build time, not calendar time. Hours of Done tasks are the original estimates, not measured time. Integration and milestone rows (owner All) carry no hours and are excluded from Team Load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>Blue text = inputs you can change. Black = formulas.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>4.</t>
+          <t>1.</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>T19 is stretch: drop it first. Cut order after that: rec_product and customer_360, the SQL checks beyond the five key ones, Power BI pages beyond Campaign and Funnel. Never cut: attribution (T13), campaign summaries (T12), Grafana (G2) and the failure demo (G3).</t>
+          <t>Productive hours per member per day: 6 (blue input on Team Load sheet).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>5.</t>
+          <t>2.</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Spark runs in Docker (Python 3.11 and Java 17 are inside the image); the host needs Python 3.11 only. Status column is an input (blue): Done, In progress, To do.</t>
+          <t>Hours are focused build time, not calendar time. Hours of Done tasks are the original estimates, not measured time. Integration and milestone rows (owner All) carry no hours and are excluded from Team Load.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>6.</t>
+          <t>3.</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>T0 was a human step: Databricks workspace, SQL warehouse and token. The token stays in .env only.</t>
+          <t>Blue text = inputs you can change. Black = formulas.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>7.</t>
+          <t>4.</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Decision date 10 Oct: batch entry point is a Python script (T15). The Airflow DAG exists for the daily ad report only.</t>
+          <t>T19 is stretch: drop it first. Cut order after that: rec_product and customer_360, the SQL checks beyond the five key ones, Power BI pages beyond Campaign and Funnel. Never cut: attribution (T13), campaign summaries (T12), Grafana (G2) and the failure demo (G3).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>8.</t>
+          <t>5.</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Tasks C1-C4, AD, D1, D2, DEMO, G1, G2 were added after the 4 Oct plan (external review, address and tracking URL, live monitoring).</t>
+          <t>Spark runs in Docker (Python 3.11 and Java 17 are inside the image); the host needs Python 3.11 only. Status column is an input (blue): Done, In progress, To do.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>9.</t>
+          <t>6.</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>10 Oct: rows SPD, ALR and INV0-INV6 were added after the speed measurements and the inventory spec. Hours of these rows are estimates and owners follow the area precedent; change them freely.</t>
+          <t>T0 was a human step: Databricks workspace, SQL warehouse and token. The token stays in .env only.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
+          <t>7.</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Decision date 10 Oct: batch entry point is a Python script (T15). The Airflow DAG exists for the daily ad report only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>8.</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>Tasks C1-C4, AD, D1, D2, DEMO, G1, G2 were added after the 4 Oct plan (external review, address and tracking URL, live monitoring).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>9.</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>10 Oct: rows SPD, ALR and INV0-INV6 were added after the speed measurements and the inventory spec. Hours of these rows are estimates and owners follow the area precedent; change them freely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
           <t>10.</t>
         </is>
       </c>
-      <c r="B65" s="8" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>Inventory cut order: INV6 first, then the INV5 alert, then the INV5 dashboard polish. Keep INV1-INV4 and a basic dashboard. The inventory data is simulated and is labeled as simulated.</t>
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>11.</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>10 Oct late: the live-inventory section is an express service with a hard 20-minute promise; INV8a and INV8b add it. INV7 adds the daily marts for Grafana and Power BI. Hours are estimates; owners follow the area precedent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3332,11 +3515,11 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A4)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$56,A4)</f>
         <v/>
       </c>
       <c r="C4" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A4,'Sprint Plan'!$G$4:$G$53)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$56,A4,'Sprint Plan'!$G$4:$G$56)</f>
         <v/>
       </c>
       <c r="D4" s="12">
@@ -3359,11 +3542,11 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A5)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$56,A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A5,'Sprint Plan'!$G$4:$G$53)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$56,A5,'Sprint Plan'!$G$4:$G$56)</f>
         <v/>
       </c>
       <c r="D5" s="12">
@@ -3391,11 +3574,11 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A6)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$56,A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A6,'Sprint Plan'!$G$4:$G$53)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$56,A6,'Sprint Plan'!$G$4:$G$56)</f>
         <v/>
       </c>
       <c r="D6" s="12">
@@ -3416,7 +3599,7 @@
         </is>
       </c>
       <c r="I6" s="18">
-        <f>COUNTIF('Sprint Plan'!$K$4:$K$53,"Done")</f>
+        <f>COUNTIF('Sprint Plan'!$K$4:$K$56,"Done")</f>
         <v/>
       </c>
     </row>
@@ -3427,11 +3610,11 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A7)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$56,A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A7,'Sprint Plan'!$G$4:$G$53)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$56,A7,'Sprint Plan'!$G$4:$G$56)</f>
         <v/>
       </c>
       <c r="D7" s="12">
@@ -3452,7 +3635,7 @@
         </is>
       </c>
       <c r="I7" s="18">
-        <f>COUNTIF('Sprint Plan'!$K$4:$K$53,"In progress")</f>
+        <f>COUNTIF('Sprint Plan'!$K$4:$K$56,"In progress")</f>
         <v/>
       </c>
     </row>
@@ -3463,11 +3646,11 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF('Sprint Plan'!$C$4:$C$53,A8)</f>
+        <f>COUNTIF('Sprint Plan'!$C$4:$C$56,A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>SUMIF('Sprint Plan'!$C$4:$C$53,A8,'Sprint Plan'!$G$4:$G$53)</f>
+        <f>SUMIF('Sprint Plan'!$C$4:$C$56,A8,'Sprint Plan'!$G$4:$G$56)</f>
         <v/>
       </c>
       <c r="D8" s="12">
@@ -3488,7 +3671,7 @@
         </is>
       </c>
       <c r="I8" s="18">
-        <f>COUNTIF('Sprint Plan'!$K$4:$K$53,"To do")</f>
+        <f>COUNTIF('Sprint Plan'!$K$4:$K$56,"To do")</f>
         <v/>
       </c>
     </row>
@@ -3512,7 +3695,7 @@
         </is>
       </c>
       <c r="I9" s="18">
-        <f>SUMIF('Sprint Plan'!$K$4:$K$53,"Done",'Sprint Plan'!$G$4:$G$53)</f>
+        <f>SUMIF('Sprint Plan'!$K$4:$K$56,"Done",'Sprint Plan'!$G$4:$G$56)</f>
         <v/>
       </c>
     </row>
@@ -3523,7 +3706,7 @@
         </is>
       </c>
       <c r="I10" s="18">
-        <f>SUM('Sprint Plan'!$G$4:$G$53)</f>
+        <f>SUM('Sprint Plan'!$G$4:$G$56)</f>
         <v/>
       </c>
     </row>
@@ -3549,7 +3732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6321,8 +6504,203 @@
         <v/>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="8">
+        <f>'Sprint Plan'!A54</f>
+        <v/>
+      </c>
+      <c r="B54" s="8">
+        <f>'Sprint Plan'!B54</f>
+        <v/>
+      </c>
+      <c r="C54" s="8">
+        <f>'Sprint Plan'!C54</f>
+        <v/>
+      </c>
+      <c r="D54" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D54,D$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="E54" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D54,E$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="F54" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D54,F$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="G54" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D54,G$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="H54" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D54,H$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="I54" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D54,I$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="J54" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D54,J$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="K54" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D54,K$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="L54" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D54,L$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+      <c r="M54" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D54,M$3&lt;='Sprint Plan'!$E54),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8">
+        <f>'Sprint Plan'!A55</f>
+        <v/>
+      </c>
+      <c r="B55" s="8">
+        <f>'Sprint Plan'!B55</f>
+        <v/>
+      </c>
+      <c r="C55" s="8">
+        <f>'Sprint Plan'!C55</f>
+        <v/>
+      </c>
+      <c r="D55" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D55,D$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="E55" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D55,E$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="F55" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D55,F$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D55,G$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="H55" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D55,H$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="I55" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D55,I$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="J55" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D55,J$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="K55" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D55,K$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="L55" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D55,L$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+      <c r="M55" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D55,M$3&lt;='Sprint Plan'!$E55),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8">
+        <f>'Sprint Plan'!A56</f>
+        <v/>
+      </c>
+      <c r="B56" s="8">
+        <f>'Sprint Plan'!B56</f>
+        <v/>
+      </c>
+      <c r="C56" s="8">
+        <f>'Sprint Plan'!C56</f>
+        <v/>
+      </c>
+      <c r="D56" s="21">
+        <f>IF(AND(D$3&gt;='Sprint Plan'!$D56,D$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="E56" s="21">
+        <f>IF(AND(E$3&gt;='Sprint Plan'!$D56,E$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="F56" s="21">
+        <f>IF(AND(F$3&gt;='Sprint Plan'!$D56,F$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="G56" s="21">
+        <f>IF(AND(G$3&gt;='Sprint Plan'!$D56,G$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="H56" s="21">
+        <f>IF(AND(H$3&gt;='Sprint Plan'!$D56,H$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="I56" s="21">
+        <f>IF(AND(I$3&gt;='Sprint Plan'!$D56,I$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="J56" s="21">
+        <f>IF(AND(J$3&gt;='Sprint Plan'!$D56,J$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="K56" s="21">
+        <f>IF(AND(K$3&gt;='Sprint Plan'!$D56,K$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="L56" s="21">
+        <f>IF(AND(L$3&gt;='Sprint Plan'!$D56,L$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+      <c r="M56" s="21">
+        <f>IF(AND(M$3&gt;='Sprint Plan'!$D56,M$3&lt;='Sprint Plan'!$E56),1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
   </sheetData>
-  <conditionalFormatting sqref="D4:M53">
+  <conditionalFormatting sqref="D4:M56">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(D4=1,LEFT($A4,1)="M")</formula>
     </cfRule>

</xml_diff>

<commit_message>
Update the sprint sheet to 11 October
Mark INV1 to INV8b Done with the commits and the checks run on 11 October,
set the header date, keep G3, T17 and T18 open with their reasons, and add
assumption 12 with the Spark test result so far.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W2R5vwQjBqqR6BPgWnVBe9
</commit_message>
<xml_diff>
--- a/docs/FunnelStream-Sprint-Plan-v3.xlsx
+++ b/docs/FunnelStream-Sprint-Plan-v3.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Status as of Saturday 10 October 2026. Dates of Done tasks are actual (commit history); dates of open tasks are planned.</t>
+          <t>Status as of Sunday 11 October 2026. Dates of Done tasks are actual (commit history); dates of open tasks are planned.</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Parked 10 Oct: two attempts ended when the Docker WSL VM restarted (21:52 and 22:05) and the PC clock jumped days on sleep and resume. Code, speed and alerts are done. Retry Mon 12 Oct after the PC checks; fallback: a recorded run plus the Spark replay tests</t>
+          <t>Parked 10 Oct: two attempts ended when the Docker WSL VM restarted. Code, speed and alerts are done. Not retried on 11 Oct (RAM 2 to 4 GB free here); fallback: a recorded run plus the Spark replay tests</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Samples and README done and verified; benchmark script verified, real run pending (recreates Kafka)</t>
+          <t>Samples and README done and verified; benchmark script verified, real run pending (recreates Kafka, needs owner approval)</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2588,10 +2588,10 @@
         </is>
       </c>
       <c r="D43" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="E43" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="F43" s="3">
         <f>E43-D43+1</f>
@@ -2612,12 +2612,12 @@
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Standard envelope with payload; explicit stock branch; tests first</t>
+          <t>Standard envelope with payload; explicit stock branch; committed e97d2a5. Verified 11 Oct on a clean run: Bronze and Silver take the stock topic</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="D44" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="E44" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="F44" s="3">
         <f>E44-D44+1</f>
@@ -2662,12 +2662,12 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Seeded, never negative, 8 stores, oversold lines recorded; express orders in INV8a</t>
+          <t>Seeded, never negative, 8 stores, oversold lines recorded; committed e97d2a5. Verified 11 Oct on a clean run: hero stock-out reached with --hero-units 4 (12 units was too many for 3,000 events)</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2688,10 +2688,10 @@
         </is>
       </c>
       <c r="D45" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="E45" s="17" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="F45" s="3">
         <f>E45-D45+1</f>
@@ -2712,12 +2712,12 @@
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>Adds MERGEs to a batch that SPD made faster</t>
+          <t>Silver stock tables, DDL, routing; committed e97d2a5. Verified 11 Oct on a clean run: silver_stock_* filled from the 10 Oct batches</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
         <v>46306</v>
       </c>
       <c r="E46" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F46" s="3">
         <f>E46-D46+1</f>
@@ -2762,12 +2762,12 @@
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>live_stock_now, live_oos_demand_minute, dim_store</t>
+          <t>Committed b1dea57. Verified 11 Oct on a clean run: 15 live tables via apply_live_ddl.py, live_stock_now 1,552 rows, live_oos_demand_minute and live_express_orders filled</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2788,10 +2788,10 @@
         </is>
       </c>
       <c r="D47" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="E47" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F47" s="3">
         <f>E47-D47+1</f>
@@ -2812,12 +2812,12 @@
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>7 panels, one alert</t>
+          <t>Committed b1dea57. Verified 11 Oct on a clean run: all 12 panels of the Operations dashboard return data; fs-oos-demand not asserted on the simulated run</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2838,10 +2838,10 @@
         </is>
       </c>
       <c r="D48" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="E48" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F48" s="3">
         <f>E48-D48+1</f>
@@ -2862,12 +2862,12 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>Cut first among the inventory rows</t>
+          <t>Committed b1dea57. D-1 mart built for 10 Oct (spend, ROAS, exposed spend, products at risk). The out-of-stock demand of 10 Oct is MOCK rows; 11 Oct needs its ad report first</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
         <v>46306</v>
       </c>
       <c r="E49" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F49" s="3">
         <f>E49-D49+1</f>
@@ -2912,12 +2912,12 @@
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>inventory_daily, oos_demand_daily, express_daily; second Grafana dashboard; Power BI reads the same tables</t>
+          <t>Committed b1dea57. Verified 11 Oct on a clean run: inventory_daily, oos_demand_daily, express_daily built; all 10 panels of the daily dashboard return data. Power BI tables not opened in Power BI Desktop</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2962,12 +2962,12 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>service and promised_minutes on the order; express orders take 8 to 17.5 min and never over 19.5; noise protected</t>
+          <t>Committed b1dea57. Verified 11 Oct on a clean run: express orders flow to Silver and live_express_orders (all on time at the 20-minute promise)</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2988,10 +2988,10 @@
         </is>
       </c>
       <c r="D51" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="E51" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F51" s="3">
         <f>E51-D51+1</f>
@@ -3012,12 +3012,12 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>fs-express-sla fires on any breach; rehearsal flags shorten the promise and make every Kth order late</t>
+          <t>Committed b1dea57. Express panels return data; the fs-express-sla breach path was not fired on this machine</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3267,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
@@ -3407,26 +3406,18 @@
         </is>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>12.</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>11 Oct: INV1-INV8b marked Done after real runs of the whole chain on a second PC (simulator, Kafka, Bronze, Silver, Databricks publish and Gold with 63 checks, 15 live tables, 4 Grafana dashboards, the D-1 and daily marts). Not done: Power BI Desktop (T18), failure demo (G3), real benchmark (T17). Spark tests in Docker, 11 Oct: the first full run reached 568 passed, 0 failed, then 10 setup errors in test_gold_build_spark.py while the 4 GB container sat at its memory limit (3.9 GB used; no out-of-memory error was seen); that file alone passes (23 passed, 5 min 31 s). The test files sorted after it are run separately. The inventory, express and live-sink Spark tests passed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3732,7 +3723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M89"/>
+  <dimension ref="A1:M56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6666,39 +6657,6 @@
         <v/>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
   </sheetData>
   <conditionalFormatting sqref="D4:M56">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">

</xml_diff>

<commit_message>
Mark T17 Done in the sprint sheet and update the T18 and M2 notes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W2R5vwQjBqqR6BPgWnVBe9
</commit_message>
<xml_diff>
--- a/docs/FunnelStream-Sprint-Plan-v3.xlsx
+++ b/docs/FunnelStream-Sprint-Plan-v3.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2391,7 +2391,7 @@
         <v>46306</v>
       </c>
       <c r="E39" s="17" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F39" s="3">
         <f>E39-D39+1</f>
@@ -2412,12 +2412,12 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Samples and README done and verified; benchmark script verified, real run pending (recreates Kafka, needs owner approval)</t>
+          <t>Samples and README done and verified. Benchmark recorded 11 Oct in docs/benchmark.md: 400,000 events (409,133 Kafka messages) in 388.6 s through all eight stages, 64 checks run and 0 failed. The 1 to 2 million event run was not attempted on this PC (Spark container capped at 4 GB, about 2 GB RAM and 11 GB disk free)</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Power BI Desktop downloading; model v2 with inventory and express pages in dashboards/powerbi (MODEL.md, measures.dax)</t>
+          <t>Generator extended 11 Oct to the full version 2 model: 15 tables (7 Gold, 7 Postgres marts, measures), 22 relationships, 84 measures, 5 page shells; both schema errors Power BI Desktop reported are fixed and scripts/validate_pbip.py checks every JSON file. Still to do by hand in Power BI Desktop: sign in, Refresh, build the visuals</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t>Team session</t>
+          <t>Team session. Benchmark part done on 11 Oct (400,000 events, docs/benchmark.md); failure demo (G3) and the 1 to 2 million event run are still open</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr">
@@ -3267,6 +3267,7 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
@@ -3414,10 +3415,29 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>11 Oct: INV1-INV8b marked Done after real runs of the whole chain on a second PC (simulator, Kafka, Bronze, Silver, Databricks publish and Gold with 63 checks, 15 live tables, 4 Grafana dashboards, the D-1 and daily marts). Not done: Power BI Desktop (T18), failure demo (G3), real benchmark (T17). Spark tests in Docker, 11 Oct: the first full run reached 568 passed, 0 failed, then 10 setup errors in test_gold_build_spark.py while the 4 GB container sat at its memory limit (3.9 GB used; no out-of-memory error was seen); that file alone passes (23 passed, 5 min 31 s). The test files sorted after it are run separately. The inventory, express and live-sink Spark tests passed.</t>
-        </is>
-      </c>
-    </row>
+          <t>11 Oct: INV1-INV8b marked Done after real runs of the whole chain on a second PC (simulator, Kafka, Bronze, Silver, Databricks publish and Gold with 63 checks, 15 live tables, 4 Grafana dashboards, the D-1 and daily marts). Not done: the Power BI visuals (T18), failure demo (G3), the 1 to 2 million event benchmark. The benchmark found and fixed two bugs: the simulator crashed when its manifest folder was missing, and the scratch Silver mirror tables kept rows of the previous run. Spark tests in Docker, 11 Oct: the first full run reached 568 passed, 0 failed, then 10 setup errors in test_gold_build_spark.py while the 4 GB container sat at its memory limit (3.9 GB used; no out-of-memory error was seen); that file alone passes (23 passed, 5 min 31 s). The test files sorted after it are run separately. The inventory, express and live-sink Spark tests passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark G3, T17, T18, T19 and M2 Done in the sprint sheet
The failure demo ran with both alerts and zero duplicates, the benchmark ran at
400,000 and 1,000,000 events, Power BI opened in Desktop with 8 pages, and
Customer 360 is built on Databricks. DOC, M3 and M4 remain.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W2R5vwQjBqqR6BPgWnVBe9
</commit_message>
<xml_diff>
--- a/docs/FunnelStream-Sprint-Plan-v3.xlsx
+++ b/docs/FunnelStream-Sprint-Plan-v3.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Status as of Sunday 11 October 2026. Dates of Done tasks are actual (commit history); dates of open tasks are planned.</t>
+          <t>Status as of Monday 12 October 2026. Dates of Done tasks are actual (commit history); dates of open tasks are planned.</t>
         </is>
       </c>
     </row>
@@ -2362,12 +2362,12 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Parked 10 Oct: two attempts ended when the Docker WSL VM restarted. Code, speed and alerts are done. Not retried on 11 Oct (RAM 2 to 4 GB free here); fallback: a recorded run plus the Spark replay tests</t>
+          <t>Run for real on 12 Oct (docs/RUNNING.md): zero duplicate keys in 7 Silver tables before the crash; docker kill at 00:07:27; the Silver-silent alert fired at 00:10:14 (+2 m 47 s) and No-events at 00:11:15 (+3 m 48 s); restart at 00:13:55, heartbeat back and both alerts resolved by 00:17:17; zero duplicates again after the replay (silver_events 44,536 to 56,710 rows)</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Samples and README done and verified. Benchmark recorded 11 Oct in docs/benchmark.md: 400,000 events (409,133 Kafka messages) in 388.6 s through all eight stages, 64 checks run and 0 failed. The 1 to 2 million event run was not attempted on this PC (Spark container capped at 4 GB, about 2 GB RAM and 11 GB disk free)</t>
+          <t>Samples and README done and verified. Benchmark recorded in docs/benchmark.md: 400,000 events in 388.6 s on 11 Oct and 1,000,000 events (1,022,333 Kafka messages) in 654.7 s on 12 Oct, all eight stages, 64 checks run and 0 failed. Two bugs found and fixed by the runs: the simulator crashed when its manifest folder was missing, and the scratch Silver mirror kept rows of the previous run</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2462,12 +2462,12 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Generator extended 11 Oct to the full version 2 model: 15 tables (7 Gold, 7 Postgres marts, measures), 22 relationships, 84 measures, 5 page shells; both schema errors Power BI Desktop reported are fixed and scripts/validate_pbip.py checks every JSON file. Still to do by hand in Power BI Desktop: sign in, Refresh, build the visuals</t>
+          <t>Power BI Desktop opened and loaded the generated project on 12 Oct (after fixing the schema errors, the boolean filter, the DAX reserved word and the auto date tables). 8 pages, 112 visuals, 19 tables, 104 measures, custom theme with the validated palette. The committed project is Desktop's saved version</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2512,12 +2512,12 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Cut first if late</t>
+          <t>Gold customer_360 built (step 13, recomputed in full, 5,000 rows on Databricks, 65 checks 0 failed), 5 hand-built Spark tests plus the end-to-end and checks suites, sample exported, Power BI table, 8 measures and a Customer 360 page</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3162,12 +3162,12 @@
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t>Team session. Benchmark part done on 11 Oct (400,000 events, docs/benchmark.md); failure demo (G3) and the 1 to 2 million event run are still open</t>
+          <t>Failure demo (G3) passed, 1,000,000-event run done and the benchmark recorded (docs/benchmark.md). Run on one PC by one person, not as a team session</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3419,18 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>13.</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>12 Oct: G3, T17, T18, T19 and M2 marked Done after real runs (failure demo with both alerts, 400k and 1,000,000 event benchmarks, Power BI opened in Desktop, Customer 360 built on Databricks). Still To do: DOC (refresh of the deck, PDF and README screenshots), M3 (rehearsal) and M4 (defense), which need people. The hour figures are the original estimates.</t>
+        </is>
+      </c>
+    </row>
     <row r="72"/>
     <row r="73"/>
     <row r="74"/>
@@ -3438,6 +3449,11 @@
     <row r="87"/>
     <row r="88"/>
     <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>